<commit_message>
Write data back to excel
</commit_message>
<xml_diff>
--- a/vtiger-crm-am147/src/test/resources/testScriptData.xlsx
+++ b/vtiger-crm-am147/src/test/resources/testScriptData.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="org" sheetId="1" r:id="rId1"/>
+    <sheet name="contact" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -19,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="18">
   <si>
     <t>orgName</t>
   </si>
@@ -52,6 +53,27 @@
   </si>
   <si>
     <t>sunny_dev_</t>
+  </si>
+  <si>
+    <t>lastName</t>
+  </si>
+  <si>
+    <t>Kumar</t>
+  </si>
+  <si>
+    <t>Sinha</t>
+  </si>
+  <si>
+    <t>Something</t>
+  </si>
+  <si>
+    <t>phoneNum</t>
+  </si>
+  <si>
+    <t>9876543210</t>
+  </si>
+  <si>
+    <t>TRUE</t>
   </si>
 </sst>
 </file>
@@ -108,11 +130,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -393,69 +416,183 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.42578125" customWidth="1"/>
+    <col min="2" max="2" width="17.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B1" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B2" s="1">
+        <v>9876543210</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B3" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B4" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B5" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B6" s="1"/>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B7" s="1"/>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B8" s="1"/>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B9" s="1"/>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B10" s="1"/>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>10</v>
       </c>
+      <c r="B11" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:H7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
+      <c r="H5" s="1"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="1"/>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1"/>
+      <c r="H7" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>